<commit_message>
Add MCP framework updates
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t>wrongpassword</t>
   </si>
@@ -57,21 +57,6 @@
   </si>
   <si>
     <t>personal</t>
-  </si>
-  <si>
-    <t>Meeting</t>
-  </si>
-  <si>
-    <t>Time sync at 10 AM</t>
-  </si>
-  <si>
-    <t>work</t>
-  </si>
-  <si>
-    <t>Idea</t>
-  </si>
-  <si>
-    <t>Build AI project</t>
   </si>
 </sst>
 </file>
@@ -378,6 +363,8 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
         <v>8</v>
       </c>
@@ -416,28 +403,6 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>